<commit_message>
Fixed formatting for VIF tables
</commit_message>
<xml_diff>
--- a/notebooks/extra_analysis/ema_rwd_final_statistics_tables_logit_vif_due_protocol.xlsx
+++ b/notebooks/extra_analysis/ema_rwd_final_statistics_tables_logit_vif_due_protocol.xlsx
@@ -536,20 +536,28 @@
           <t>431 (62.9)</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>1.047125979413853</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="n">
-        <v>1.202252637901109</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.8360685567356473</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.196074163947043</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -567,20 +575,28 @@
           <t>89 (60.1)</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1.047125979413853</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
-      <c r="G4" t="n">
-        <v>1.202252637901109</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.9208564154930813</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1.085945629715291</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -623,20 +639,28 @@
           <t>185 (70.9)</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>1.090497665655317</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
-      <c r="G6" t="n">
-        <v>1.189185158799696</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.8411323647642058</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1.188873525607744</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -679,20 +703,28 @@
           <t>33 (55.0)</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>1.117159217367746</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
       </c>
       <c r="F8" t="n">
         <v>4</v>
       </c>
-      <c r="G8" t="n">
-        <v>2.426166405668426</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.7421209561872248</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1.347489235633061</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2.43</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.74</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -710,20 +742,28 @@
           <t>18 (64.3)</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>1.117159217367746</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
       </c>
       <c r="F9" t="n">
         <v>4</v>
       </c>
-      <c r="G9" t="n">
-        <v>2.426166405668426</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.937927365847562</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1.066180640860549</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2.43</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -741,20 +781,28 @@
           <t>219 (56.0)</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>1.117159217367746</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
       </c>
       <c r="F10" t="n">
         <v>4</v>
       </c>
-      <c r="G10" t="n">
-        <v>2.426166405668426</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.6139975456647532</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.628671005382173</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2.43</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.61</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -772,20 +820,28 @@
           <t>15 (41.7)</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>1.117159217367746</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
       </c>
       <c r="F11" t="n">
         <v>4</v>
       </c>
-      <c r="G11" t="n">
-        <v>2.426166405668426</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.9080840131285497</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1.101219695031057</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2.43</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -828,20 +884,28 @@
           <t>1139 (59.4)</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>1.059537897941724</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="n">
-        <v>1.122620557174767</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.8906970691041618</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1.122716167692987</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -884,20 +948,28 @@
           <t>126 (53.6)</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>1.156362727783047</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" t="n">
-        <v>1.33717475820585</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.7473354834681465</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1.338087140408907</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -919,20 +991,28 @@
           <t>611 (64.7)</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>1.130627998991962</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="n">
-        <v>1.278319672104568</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.7821205680347225</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.278575248970571</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.78</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -975,20 +1055,28 @@
           <t>293 (48.0)</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>1.07163249087097</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F18" t="n">
         <v>3</v>
       </c>
-      <c r="G18" t="n">
-        <v>1.514520775534277</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.5591420206054732</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1.788454387522402</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1.79</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1006,20 +1094,28 @@
           <t>349 (57.8)</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>1.07163249087097</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F19" t="n">
         <v>3</v>
       </c>
-      <c r="G19" t="n">
-        <v>1.514520775534277</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.540625424716542</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1.849709529521878</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1037,20 +1133,28 @@
           <t>380 (67.1)</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>1.07163249087097</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F20" t="n">
         <v>3</v>
       </c>
-      <c r="G20" t="n">
-        <v>1.514520775534277</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.5350804229037862</v>
-      </c>
-      <c r="I20" t="n">
-        <v>1.868877942820591</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1114,20 +1218,28 @@
           <t>329 (57.8)</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>1.065896422820478</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F23" t="n">
         <v>4</v>
       </c>
-      <c r="G23" t="n">
-        <v>1.666172789437331</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.5860589489362312</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1.706312994307352</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>0.59</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1145,20 +1257,28 @@
           <t>140 (57.4)</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>1.065896422820478</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F24" t="n">
         <v>4</v>
       </c>
-      <c r="G24" t="n">
-        <v>1.666172789437331</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.7352866087189864</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1.360013888655196</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>0.74</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1176,20 +1296,28 @@
           <t>155 (59.6)</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>1.065896422820478</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F25" t="n">
         <v>4</v>
       </c>
-      <c r="G25" t="n">
-        <v>1.666172789437331</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.6870344670372789</v>
-      </c>
-      <c r="I25" t="n">
-        <v>1.45553105117467</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>0.69</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1207,20 +1335,28 @@
           <t>467 (64.1)</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>1.065896422820478</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F26" t="n">
         <v>4</v>
       </c>
-      <c r="G26" t="n">
-        <v>1.666172789437331</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.4478223352204873</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2.233028416297382</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2.23</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1263,20 +1399,28 @@
           <t>298 (64.5)</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>1.07007998891346</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F28" t="n">
         <v>4</v>
       </c>
-      <c r="G28" t="n">
-        <v>1.719214006452929</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.5852085301513458</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1.708792590124039</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>0.59</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1294,20 +1438,28 @@
           <t>257 (56.2)</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>1.07007998891346</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F29" t="n">
         <v>4</v>
       </c>
-      <c r="G29" t="n">
-        <v>1.719214006452929</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.5520649792939719</v>
-      </c>
-      <c r="I29" t="n">
-        <v>1.811380974172435</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1325,20 +1477,28 @@
           <t>280 (60.9)</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>1.07007998891346</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F30" t="n">
         <v>4</v>
       </c>
-      <c r="G30" t="n">
-        <v>1.719214006452929</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0.4408184309222378</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2.268507688999973</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>0.44</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1356,20 +1516,28 @@
           <t>239 (51.8)</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>1.07007998891346</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F31" t="n">
         <v>4</v>
       </c>
-      <c r="G31" t="n">
-        <v>1.719214006452929</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0.5168951378050163</v>
-      </c>
-      <c r="I31" t="n">
-        <v>1.934628374038258</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>0.52</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1391,20 +1559,28 @@
           <t>76 (67.9)</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v>1.072582580534232</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F32" t="n">
         <v>5</v>
       </c>
-      <c r="G32" t="n">
-        <v>2.0151500723723</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0.8272108017543004</v>
-      </c>
-      <c r="I32" t="n">
-        <v>1.208881699657764</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>0.83</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1422,20 +1598,28 @@
           <t>21 (63.6)</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>1.072582580534232</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F33" t="n">
         <v>5</v>
       </c>
-      <c r="G33" t="n">
-        <v>2.0151500723723</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0.919101502837118</v>
-      </c>
-      <c r="I33" t="n">
-        <v>1.088019110961261</v>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1453,20 +1637,28 @@
           <t>419 (67.0)</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>1.072582580534232</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F34" t="n">
         <v>5</v>
       </c>
-      <c r="G34" t="n">
-        <v>2.0151500723723</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.6674579935868298</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1.498221625343243</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1484,20 +1676,28 @@
           <t>87 (67.4)</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>1.072582580534232</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F35" t="n">
         <v>5</v>
       </c>
-      <c r="G35" t="n">
-        <v>2.0151500723723</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.8812417191474186</v>
-      </c>
-      <c r="I35" t="n">
-        <v>1.134762436085615</v>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1536,20 +1736,28 @@
           <t>52 (47.7)</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>1.072582580534232</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F37" t="n">
         <v>5</v>
       </c>
-      <c r="G37" t="n">
-        <v>2.0151500723723</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.8230747894336256</v>
-      </c>
-      <c r="I37" t="n">
-        <v>1.214956420531505</v>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>0.82</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1571,20 +1779,28 @@
           <t>375 (59.3)</t>
         </is>
       </c>
-      <c r="E38" t="n">
-        <v>1.068963374996803</v>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
-      <c r="G38" t="n">
-        <v>1.142682697084556</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0.8750558059440814</v>
-      </c>
-      <c r="I38" t="n">
-        <v>1.142784258109251</v>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1627,20 +1843,28 @@
           <t>10 (31.2)</t>
         </is>
       </c>
-      <c r="E40" t="n">
-        <v>1.032711815864797</v>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
       </c>
       <c r="F40" t="n">
         <v>2</v>
       </c>
-      <c r="G40" t="n">
-        <v>1.13740880067865</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.9325747493539489</v>
-      </c>
-      <c r="I40" t="n">
-        <v>1.07230010322793</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1679,20 +1903,28 @@
           <t>16 (36.4)</t>
         </is>
       </c>
-      <c r="E42" t="n">
-        <v>1.032711815864797</v>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
       </c>
       <c r="F42" t="n">
         <v>2</v>
       </c>
-      <c r="G42" t="n">
-        <v>1.13740880067865</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.9402583200227908</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1.063537518046914</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1735,20 +1967,28 @@
           <t>340 (41.7)</t>
         </is>
       </c>
-      <c r="E44" t="n">
-        <v>1.18294602136324</v>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
-      <c r="G44" t="n">
-        <v>1.399361289459119</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.7148273854095196</v>
-      </c>
-      <c r="I44" t="n">
-        <v>1.398939129097729</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>0.71</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1791,20 +2031,28 @@
           <t>485 (65.4)</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v>1.173135608594766</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
       </c>
       <c r="F46" t="n">
         <v>1</v>
       </c>
-      <c r="G46" t="n">
-        <v>1.376247156153012</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.727592396726763</v>
-      </c>
-      <c r="I46" t="n">
-        <v>1.374395890472088</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>